<commit_message>
Recognize SurveyMonkey exports and read their two header rows (v0.7, step 2, D-044, D-048)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exemples/bases-fictives/travail-t2_surveymonkey.xlsx
+++ b/exemples/bases-fictives/travail-t2_surveymonkey.xlsx
@@ -419,47 +419,47 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Respondent ID</t>
+          <t>respondent_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Collector ID</t>
+          <t>collector_id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>date_created</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>End Date</t>
+          <t>date_modified</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>IP Address</t>
+          <t>ip_address</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Email Address</t>
+          <t>email_address</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>First Name</t>
+          <t>first_name</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Last Name</t>
+          <t>last_name</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Custom Data 1</t>
+          <t>custom_1</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">

</xml_diff>